<commit_message>
baro works, battery voltage works, horizon exists
</commit_message>
<xml_diff>
--- a/Software/Witness/softwarev1/AMA comms standard.xlsx
+++ b/Software/Witness/softwarev1/AMA comms standard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ejfso\Documents\GitHub\witness\Software\Witness\softwarev1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3F857A9-9C0F-4D14-B983-1B018BA6BCB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49B7C6C8-F1E7-4447-A676-7A3B87535FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="18700" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="18700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fields" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="97">
   <si>
     <t>Field</t>
   </si>
@@ -136,9 +136,6 @@
     <t>Sensors</t>
   </si>
   <si>
-    <t>status, uptime, accel, gyro</t>
-  </si>
-  <si>
     <t>Just high rate sensor data, 10hz down</t>
   </si>
   <si>
@@ -148,9 +145,6 @@
     <t>State</t>
   </si>
   <si>
-    <t>Status, uptime, Orientation, position, Velocity, Lat/lon, GPS alt</t>
-  </si>
-  <si>
     <t>Estimated state and gps state, 2hz?</t>
   </si>
   <si>
@@ -160,9 +154,6 @@
     <t>Camera</t>
   </si>
   <si>
-    <t>FC status, FC uptime, IRIS status, IRIS uptime, current sense</t>
-  </si>
-  <si>
     <t>Camera sense data, 1hz</t>
   </si>
   <si>
@@ -238,9 +229,6 @@
     <t>Source board</t>
   </si>
   <si>
-    <t>Root source</t>
-  </si>
-  <si>
     <t>Category</t>
   </si>
   <si>
@@ -275,13 +263,79 @@
   </si>
   <si>
     <t>witness mcu temp</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> IRIS status, IRIS uptime, 4x current sense</t>
+  </si>
+  <si>
+    <t>ground station status, ground station Uptime</t>
+  </si>
+  <si>
+    <t>fc status, fc uptime, 3x filtered accel,3x gyro,</t>
+  </si>
+  <si>
+    <t>MS5607 Alt</t>
+  </si>
+  <si>
+    <t>0x05</t>
+  </si>
+  <si>
+    <t>Command</t>
+  </si>
+  <si>
+    <t>Status, uptime, command</t>
+  </si>
+  <si>
+    <t>command</t>
+  </si>
+  <si>
+    <t>general</t>
+  </si>
+  <si>
+    <t>Any</t>
+  </si>
+  <si>
+    <t>fc Status, fc uptime, Orientation quaternion , position vector, Velocity vector, Lat/lon, GPS alt, baro alt, FC battery voltage</t>
+  </si>
+  <si>
+    <t>FC status, FC uptime, IRIS status, IRIS uptime, current sense, IRIS battery voltage</t>
+  </si>
+  <si>
+    <t>sending commands from the ground station to the board</t>
+  </si>
+  <si>
+    <t>ms</t>
+  </si>
+  <si>
+    <t>100 mV/count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">float multiplied by 10000 </t>
+  </si>
+  <si>
+    <t>unix time stamp</t>
+  </si>
+  <si>
+    <t>Discrete bits</t>
+  </si>
+  <si>
+    <t>format (compressed)</t>
+  </si>
+  <si>
+    <t>data type</t>
+  </si>
+  <si>
+    <t>unsigned integer</t>
+  </si>
+  <si>
+    <t>16 bit flags that can be set</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -306,6 +360,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="5">
@@ -372,7 +438,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -398,6 +464,23 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -698,23 +781,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M48"/>
-  <sheetFormatPr defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:M51"/>
+  <sheetFormatPr defaultRowHeight="20" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="26.453125" customWidth="1"/>
     <col min="3" max="3" width="21.36328125" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="7" max="7" width="20.453125" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="8" max="8" width="22.36328125" customWidth="1"/>
+    <col min="9" max="9" width="22.54296875" customWidth="1"/>
     <col min="12" max="12" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>21</v>
@@ -724,26 +808,28 @@
         <v>22</v>
       </c>
       <c r="G1" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="L1" t="s">
+        <v>63</v>
+      </c>
+      <c r="M1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="20" customHeight="1" thickBot="1">
+      <c r="A2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="H1" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="I1" s="7"/>
-      <c r="L1" t="s">
-        <v>67</v>
-      </c>
-      <c r="M1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>69</v>
-      </c>
       <c r="C2" s="2">
         <v>2</v>
       </c>
@@ -757,22 +843,28 @@
         <v>1</v>
       </c>
       <c r="G2" t="str">
-        <f t="shared" ref="G2:G43" si="0">VLOOKUP(B2,L:M,2,FALSE)</f>
-        <v>Witness</v>
+        <f t="shared" ref="G2:G37" si="0">VLOOKUP(B2,L:M,2,FALSE)</f>
+        <v>Witness</v>
+      </c>
+      <c r="H2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I2" t="s">
+        <v>96</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A3" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C3" s="2">
         <v>4</v>
@@ -790,37 +882,43 @@
         <f t="shared" si="0"/>
         <v>Witness</v>
       </c>
+      <c r="H3" t="s">
+        <v>95</v>
+      </c>
+      <c r="I3" t="s">
+        <v>88</v>
+      </c>
       <c r="L3" s="9" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="M3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A4" s="5" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G4" t="str">
         <f t="shared" si="0"/>
         <v>Witness</v>
       </c>
       <c r="L4" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="M4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A5" s="5" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C5" s="6">
         <v>2</v>
@@ -838,19 +936,22 @@
         <f t="shared" si="0"/>
         <v>Witness</v>
       </c>
+      <c r="I5" s="17" t="s">
+        <v>89</v>
+      </c>
       <c r="L5" t="s">
+        <v>67</v>
+      </c>
+      <c r="M5" t="s">
         <v>71</v>
       </c>
-      <c r="M5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="6" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A6" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C6" s="2">
         <v>4</v>
@@ -869,18 +970,18 @@
         <v>Iris</v>
       </c>
       <c r="L6" t="s">
+        <v>68</v>
+      </c>
+      <c r="M6" t="s">
         <v>72</v>
       </c>
-      <c r="M6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A7" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C7" s="2">
         <v>2</v>
@@ -898,13 +999,19 @@
         <f t="shared" si="0"/>
         <v>Iris</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A8" s="1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C8" s="2">
         <v>2</v>
@@ -922,13 +1029,19 @@
         <f t="shared" si="0"/>
         <v>Iris</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="H8" t="s">
+        <v>95</v>
+      </c>
+      <c r="I8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A9" s="5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C9" s="6">
         <v>2</v>
@@ -946,20 +1059,23 @@
         <f t="shared" si="0"/>
         <v>Iris</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="I9" s="17" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="B10" s="1"/>
       <c r="G10" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A11" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C11" s="2">
         <v>2</v>
@@ -978,12 +1094,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A12" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C12" s="2">
         <v>2</v>
@@ -1002,12 +1118,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
@@ -1026,12 +1142,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A14" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C14" s="2">
         <v>4</v>
@@ -1050,12 +1166,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A15" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C15" s="2">
         <v>4</v>
@@ -1074,12 +1190,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:13" ht="20" customHeight="1" thickBot="1">
       <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C16" s="2">
         <v>4</v>
@@ -1098,12 +1214,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="A17" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C17" s="2">
         <v>4</v>
@@ -1122,12 +1238,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C18" s="2">
         <v>4</v>
@@ -1146,12 +1262,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="A19" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C19" s="2">
         <v>4</v>
@@ -1170,12 +1286,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C20" s="2">
         <v>4</v>
@@ -1194,12 +1310,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C21" s="2">
         <v>4</v>
@@ -1218,12 +1334,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C22" s="2">
         <v>4</v>
@@ -1242,12 +1358,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="A23" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="C23" s="2">
         <v>4</v>
@@ -1266,266 +1382,266 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="B24" s="1"/>
       <c r="G24" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="B25" s="1"/>
       <c r="G25" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:7" ht="20" customHeight="1" thickBot="1">
       <c r="A26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2">
+        <v>2</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="20" customHeight="1" thickBot="1">
+      <c r="A27" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="2">
+        <v>2</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2">
+        <v>2</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G27" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="20" customHeight="1" thickBot="1">
+      <c r="A28" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" s="2">
+        <v>2</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2">
+        <v>2</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G28" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="20" customHeight="1" thickBot="1">
+      <c r="A29" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C26" s="2">
-        <v>2</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E26" s="2">
-        <v>2</v>
-      </c>
-      <c r="F26" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G26" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="1" t="s">
+      <c r="B29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C29" s="2">
+        <v>2</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2">
+        <v>2</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G29" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="20" customHeight="1" thickBot="1">
+      <c r="A30" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C27" s="2">
-        <v>2</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E27" s="2">
-        <v>2</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G27" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="1" t="s">
+      <c r="B30" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C30" s="2">
+        <v>2</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2">
+        <v>2</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G30" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="20" customHeight="1" thickBot="1">
+      <c r="A31" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C28" s="2">
-        <v>2</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E28" s="2">
-        <v>2</v>
-      </c>
-      <c r="F28" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G28" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="1" t="s">
+      <c r="B31" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" s="2">
+        <v>2</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2">
+        <v>2</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G31" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="20" customHeight="1" thickBot="1">
+      <c r="A32" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C29" s="2">
-        <v>2</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E29" s="2">
-        <v>2</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G29" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="1" t="s">
+      <c r="B32" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" s="2">
+        <v>2</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2">
+        <v>2</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G32" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A33" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C30" s="2">
-        <v>2</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E30" s="2">
-        <v>2</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G30" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="1" t="s">
+      <c r="B33" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C33" s="2">
+        <v>2</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2">
+        <v>2</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G33" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A34" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C31" s="2">
-        <v>2</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E31" s="2">
-        <v>2</v>
-      </c>
-      <c r="F31" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G31" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="1" t="s">
+      <c r="B34" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C34" s="2">
+        <v>2</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E34" s="2">
+        <v>2</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G34" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A35" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C32" s="2">
-        <v>2</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E32" s="2">
-        <v>2</v>
-      </c>
-      <c r="F32" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G32" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="1" t="s">
+      <c r="B35" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C35" s="2">
+        <v>2</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E35" s="2">
+        <v>2</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G35" t="str">
+        <f t="shared" si="0"/>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A36" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C33" s="2">
-        <v>2</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E33" s="2">
-        <v>2</v>
-      </c>
-      <c r="F33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G33" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C34" s="2">
-        <v>2</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E34" s="2">
-        <v>2</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G34" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C35" s="2">
-        <v>2</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E35" s="2">
-        <v>2</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="G35" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="1" t="s">
-        <v>58</v>
-      </c>
       <c r="B36" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C36" s="2">
         <v>3</v>
@@ -1544,12 +1660,12 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:9" ht="20" customHeight="1" thickBot="1">
       <c r="A37" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C37" s="2">
         <v>2</v>
@@ -1568,67 +1684,61 @@
         <v>Witness</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:9" ht="20" customHeight="1" thickBot="1">
       <c r="A38" s="1" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C38" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>1</v>
       </c>
       <c r="E38" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>1</v>
       </c>
       <c r="G38" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B39" s="1"/>
-      <c r="G39" t="e">
-        <f t="shared" si="0"/>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A40" s="1" t="s">
+        <f t="shared" ref="G38" si="1">VLOOKUP(B38,L:M,2,FALSE)</f>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A39" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" s="2">
+        <v>2</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E39" s="2">
+        <v>1</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="G39" t="str">
+        <f>VLOOKUP(B39,L:M,2,FALSE)</f>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="20" customHeight="1" thickBot="1"/>
+    <row r="41" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A41" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C40" s="2">
-        <v>3</v>
-      </c>
-      <c r="D40" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E40">
-        <v>3</v>
-      </c>
-      <c r="F40" t="s">
-        <v>1</v>
-      </c>
-      <c r="G40" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="B41" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="C41" s="2">
         <v>3</v>
@@ -1643,157 +1753,213 @@
         <v>1</v>
       </c>
       <c r="G41" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <f>VLOOKUP(B41,L:M,2,FALSE)</f>
+        <v>Witness</v>
+      </c>
+      <c r="I41" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="20" customHeight="1" thickBot="1">
       <c r="A42" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C42" s="2">
+        <v>3</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E42">
+        <v>3</v>
+      </c>
+      <c r="F42" t="s">
+        <v>1</v>
+      </c>
+      <c r="G42" t="str">
+        <f>VLOOKUP(B42,L:M,2,FALSE)</f>
+        <v>Witness</v>
+      </c>
+      <c r="I42" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A43" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C42" s="2">
+      <c r="B43" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C43" s="2">
         <v>4</v>
       </c>
-      <c r="D42" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E42">
+      <c r="D43" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E43">
         <v>4</v>
       </c>
-      <c r="F42" t="s">
-        <v>1</v>
-      </c>
-      <c r="G42" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A43" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C43" s="6">
+      <c r="F43" t="s">
+        <v>1</v>
+      </c>
+      <c r="G43" t="str">
+        <f>VLOOKUP(B43,L:M,2,FALSE)</f>
+        <v>Witness</v>
+      </c>
+      <c r="I43" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A44" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" s="6">
         <v>4</v>
       </c>
-      <c r="D43" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E43" s="6">
+      <c r="D44" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E44" s="6">
         <v>4</v>
       </c>
-      <c r="F43" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="G43" t="str">
-        <f t="shared" si="0"/>
-        <v>Witness</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B44" s="1"/>
-      <c r="G44" t="e">
-        <f t="shared" ref="G44:G48" si="1">VLOOKUP(B44,L:M,2,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F44" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G44" t="str">
+        <f>VLOOKUP(B44,L:M,2,FALSE)</f>
+        <v>Witness</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="20" customHeight="1" thickBot="1">
       <c r="B45" s="1"/>
       <c r="G45" t="e">
-        <f t="shared" si="1"/>
+        <f>VLOOKUP(B45,L:M,2,FALSE)</f>
         <v>#N/A</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A46" s="1" t="s">
+    <row r="46" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="B46" s="1"/>
+      <c r="G46" t="e">
+        <f>VLOOKUP(B46,L:M,2,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A47" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B46" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C46" s="2">
-        <v>1</v>
-      </c>
-      <c r="D46" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E46">
-        <v>1</v>
-      </c>
-      <c r="F46" t="s">
-        <v>1</v>
-      </c>
-      <c r="G46" t="str">
-        <f t="shared" si="1"/>
+      <c r="B47" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C47" s="2">
+        <v>1</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47" t="s">
+        <v>1</v>
+      </c>
+      <c r="G47" t="str">
+        <f>VLOOKUP(B47,L:M,2,FALSE)</f>
         <v>Iris</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A47" s="1" t="s">
+    <row r="48" spans="1:9" ht="20" customHeight="1" thickBot="1">
+      <c r="A48" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B47" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C47" s="2">
-        <v>1</v>
-      </c>
-      <c r="D47" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E47">
-        <v>1</v>
-      </c>
-      <c r="F47" t="s">
-        <v>1</v>
-      </c>
-      <c r="G47" t="str">
-        <f t="shared" si="1"/>
+      <c r="B48" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C48" s="2">
+        <v>1</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48" t="s">
+        <v>1</v>
+      </c>
+      <c r="G48" t="str">
+        <f>VLOOKUP(B48,L:M,2,FALSE)</f>
         <v>Iris</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A48" s="1" t="s">
+    <row r="49" spans="1:7" ht="20" customHeight="1" thickBot="1">
+      <c r="A49" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B48" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C48" s="2">
-        <v>1</v>
-      </c>
-      <c r="D48" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E48">
-        <v>1</v>
-      </c>
-      <c r="F48" t="s">
-        <v>1</v>
-      </c>
-      <c r="G48" t="str">
-        <f t="shared" si="1"/>
+      <c r="B49" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C49" s="2">
+        <v>1</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49" t="s">
+        <v>1</v>
+      </c>
+      <c r="G49" t="str">
+        <f>VLOOKUP(B49,L:M,2,FALSE)</f>
         <v>Iris</v>
       </c>
     </row>
+    <row r="51" spans="1:7" ht="20" customHeight="1">
+      <c r="A51" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="B51" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C51" s="12">
+        <v>2</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="E51">
+        <v>2</v>
+      </c>
+      <c r="F51" t="s">
+        <v>1</v>
+      </c>
+      <c r="G51" t="s">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B1:B1048576">
+  <conditionalFormatting sqref="B41:B1048576 B1:B39">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>$L$2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B48">
+  <conditionalFormatting sqref="B41:B49 B2:B39">
     <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="Witness upkeep">
       <formula>NOT(ISERROR(SEARCH("Witness upkeep",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B48" xr:uid="{B1DD0CD9-1BA6-472E-8138-2C9775024B6E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B41:B49 B2:B39" xr:uid="{B1DD0CD9-1BA6-472E-8138-2C9775024B6E}">
       <formula1>$L:$L</formula1>
     </dataValidation>
   </dataValidations>
@@ -1803,106 +1969,111 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5FA6CC3-BB97-431C-A392-F72DBBF71C43}">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="20" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultRowHeight="20" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="4" max="4" width="116.6328125" customWidth="1"/>
-    <col min="5" max="5" width="76.90625" customWidth="1"/>
+    <col min="1" max="1" width="8.7265625" style="13"/>
+    <col min="2" max="2" width="25" style="13" customWidth="1"/>
+    <col min="3" max="3" width="8.7265625" style="13"/>
+    <col min="4" max="4" width="143" style="13" customWidth="1"/>
+    <col min="5" max="5" width="76.90625" style="13" customWidth="1"/>
+    <col min="6" max="16384" width="8.7265625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="3" t="s">
+    <row r="1" spans="1:5" ht="20" customHeight="1" thickBot="1">
+      <c r="A1" s="13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="20" customHeight="1" thickBot="1">
+      <c r="A2" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="14" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:5" ht="20" customHeight="1" thickBot="1">
+      <c r="A3" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="3">
-        <f>SUM(Fields!E2,Fields!E3,Fields!E11:E13,Fields!E33:E35)</f>
-        <v>18</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="C3" s="14"/>
+      <c r="D3" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="3" t="s">
+    </row>
+    <row r="4" spans="1:5" ht="20" customHeight="1" thickBot="1">
+      <c r="A4" s="14" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="3" t="s">
+      <c r="B4" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="15"/>
+      <c r="D4" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="E4" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C4" s="4">
-        <f>SUM(Fields!E2,Fields!E3,Fields!E14:E17,Fields!E18:E20,Fields!E21:E23,Fields!E40:E43)</f>
-        <v>47</v>
-      </c>
-      <c r="D4" s="3" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="20" customHeight="1" thickBot="1">
+      <c r="A5" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="B5" s="15" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="4" t="s">
+      <c r="C5" s="15"/>
+      <c r="D5" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="4" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="20" customHeight="1" thickBot="1">
+      <c r="A6" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="4">
-        <f>SUM(Fields!E2,Fields!E3,Fields!E7,Fields!E6,Fields!E46:E48)</f>
-        <v>15</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="B6" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="4" t="s">
+      <c r="C6" s="15"/>
+      <c r="D6" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="4">
-        <f>SUM(Fields!E2,Fields!E3)</f>
-        <v>6</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>45</v>
+    </row>
+    <row r="7" spans="1:5" ht="25" customHeight="1">
+      <c r="A7" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1913,8 +2084,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32ACF27C-9985-491F-AFD4-C7C4F21A73F9}">
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultRowHeight="25" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultRowHeight="25" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18.90625" customWidth="1"/>
     <col min="2" max="2" width="23.1796875" customWidth="1"/>
@@ -1922,12 +2093,12 @@
     <col min="5" max="5" width="70.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:5" ht="25" customHeight="1" thickBot="1">
       <c r="A1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" customHeight="1" thickBot="1">
       <c r="A2" s="3" t="s">
         <v>25</v>
       </c>
@@ -1944,76 +2115,45 @@
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="3">
-        <f>SUM(Fields!C2,Fields!C3,Fields!C11:C13,Fields!C33:C35)</f>
-        <v>18</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="4">
-        <f>SUM(Fields!C2,Fields!C3,Fields!C14:C17,Fields!C18:C20,Fields!C21:C23,Fields!C40:C43)</f>
-        <v>60</v>
-      </c>
-      <c r="D4" s="3" t="s">
+    <row r="3" spans="1:5" ht="25" customHeight="1" thickBot="1">
+      <c r="A3" s="4" t="s">
         <v>36</v>
       </c>
+      <c r="B3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="25" customHeight="1" thickBot="1">
+      <c r="A4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="E4" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="4">
-        <f>SUM(Fields!C2,Fields!C3,Fields!C7,Fields!C6,Fields!C46:C48)</f>
-        <v>15</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="4">
-        <f>SUM(Fields!C2,Fields!C3)</f>
-        <v>6</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>45</v>
+    </row>
+    <row r="5" spans="1:5" ht="25" customHeight="1">
+      <c r="A5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>